<commit_message>
Ship portal POS, loyalty, promo, auth, and platform config across apps.
Expand admin/super-admin feature surfaces, add mail/SMS/storage modules, Prisma migrations, shared UI, and deployment/QA docs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/qa/export/excel/BUG_LOG.xlsx
+++ b/docs/qa/export/excel/BUG_LOG.xlsx
@@ -171,7 +171,7 @@
     <t>Documented gap, not a defect</t>
   </si>
   <si>
-    <t>Admin Tables placeholder</t>
+    <t>Razorpay pay-now without keys</t>
   </si>
   <si>
     <t>ID</t>
@@ -183,31 +183,13 @@
     <t>Description</t>
   </si>
   <si>
-    <t>KL-001</t>
-  </si>
-  <si>
-    <t>Admin Tables</t>
-  </si>
-  <si>
-    <t>Phase 2 placeholder UI — use Waiter + Swagger</t>
-  </si>
-  <si>
-    <t>KL-002</t>
-  </si>
-  <si>
-    <t>Admin Inventory</t>
-  </si>
-  <si>
-    <t>Phase 2 placeholder UI — use Swagger</t>
-  </si>
-  <si>
     <t>KL-003</t>
   </si>
   <si>
-    <t>POS/KDS</t>
-  </si>
-  <si>
-    <t>Local apps only on production</t>
+    <t>POS/KDS DNS</t>
+  </si>
+  <si>
+    <t>If pos/kds URLs down, use local fallback or Blocked</t>
   </si>
   <si>
     <t>KL-004</t>
@@ -222,10 +204,28 @@
     <t>KL-005</t>
   </si>
   <si>
-    <t>Gateway sync</t>
-  </si>
-  <si>
-    <t>Requires Electron app on outlet LAN</t>
+    <t>Order Display</t>
+  </si>
+  <si>
+    <t>Prefer Admin /cds launcher</t>
+  </si>
+  <si>
+    <t>KL-006</t>
+  </si>
+  <si>
+    <t>Production stock</t>
+  </si>
+  <si>
+    <t>Stock deducts only with recipe-linked batches</t>
+  </si>
+  <si>
+    <t>KL-007</t>
+  </si>
+  <si>
+    <t>Business-type nav</t>
+  </si>
+  <si>
+    <t>Banquets/Brands/Guests/Rooms N/A on restaurant</t>
   </si>
 </sst>
 </file>

</xml_diff>